<commit_message>
Updated apps master formatting
Applied table formatting and styling to apps_master.xlsx
</commit_message>
<xml_diff>
--- a/data/apps_master.xlsx
+++ b/data/apps_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DarkPatternAnalytics\dark-pattern-impact-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{496326F9-148A-4D66-B503-D754FE1971FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D950473-E90B-4153-B45A-CF24C1C1A151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4587E125-DC69-43B6-844A-53A7A464BF81}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,16 +83,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -100,23 +114,281 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -131,6 +403,18 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{39684EC0-0266-44D0-8D92-6D85B6350C6D}" name="Table1" displayName="Table1" ref="A1:C7" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+  <autoFilter ref="A1:C7" xr:uid="{39684EC0-0266-44D0-8D92-6D85B6350C6D}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{9EDE2162-6693-4202-8387-1B48397B8754}" name="app_id" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{C6CFA460-75B8-4E9F-ABC1-2645738A8438}" name="app_name" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{16EC0B91-FDEF-41E4-AB8B-CB2BA7CA1188}" name="category" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -430,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25DACB85-C3B8-4B41-9AEC-BB19780629E9}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -438,99 +722,105 @@
     <col min="3" max="3" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7" s="10">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E15" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>